<commit_message>
moving to core measurements folder
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned_Brahmleen.xlsx
+++ b/notes/coreMeasurement/coresScanned_Brahmleen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bamo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bamo\Desktop\temp_ecol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F6A34B-87DC-4A04-AA60-07DB586B3B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{648CBB02-4CC3-4DB6-BBFD-1B6BB3FE830F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AB08" sheetId="1" r:id="rId1"/>
@@ -24,17 +24,28 @@
     <sheet name="TA01" sheetId="9" r:id="rId9"/>
     <sheet name="TO04" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3803" uniqueCount="1253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3998" uniqueCount="1309">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4057,7 +4068,175 @@
     <t>Brahmleen</t>
   </si>
   <si>
-    <t>check between ring 8/9 (unclear) and 69/70 (super small ring embedded)</t>
+    <t>80+ rings; check between ring 8/9 (unclear) and 69/70 (super small ring embedded)</t>
+  </si>
+  <si>
+    <t>80+ rings</t>
+  </si>
+  <si>
+    <t>80+ rings; ring 100-101 had 2 different widths</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check ring 8/9 - possible embedded ring; </t>
+  </si>
+  <si>
+    <t>crack on ring 61; 80+ rings</t>
+  </si>
+  <si>
+    <t>28th has a crack plz check. Crack on 69th ring. 80+ rings</t>
+  </si>
+  <si>
+    <t>crack on 10th ring; 9/10th rings are not paralell and require further attention; Crack on ring 45/46-take a look; 80+ rings; Very blurry</t>
+  </si>
+  <si>
+    <t>dust (?) on 19th ring; 80+ rings</t>
+  </si>
+  <si>
+    <t>crack on ring 70</t>
+  </si>
+  <si>
+    <t>80+ rings; crack on ring 59</t>
+  </si>
+  <si>
+    <t>tip missing; crack on ring 27; 80+ rings</t>
+  </si>
+  <si>
+    <t>division on ring 12 (2 separate widths); check ring 38 (embedded ring? Crack?); crack on ring 41</t>
+  </si>
+  <si>
+    <t>crack on ring 19; crack glue on ring 27 (?); crack glue on ring 41; 80+ rings</t>
+  </si>
+  <si>
+    <t>unsure about ring 7 (might be another ring?); 80+ rings</t>
+  </si>
+  <si>
+    <t>embedded ring in ring 15(?); 80+ rings</t>
+  </si>
+  <si>
+    <t>fixed crack on ring 70; 80+ rings</t>
+  </si>
+  <si>
+    <t>80+ rings; very slanted had to use multiple points for each ring</t>
+  </si>
+  <si>
+    <t>fixed crack on ring 50</t>
+  </si>
+  <si>
+    <t>check ring 56 (crack/unclear ring boundary)</t>
+  </si>
+  <si>
+    <t>fixed crack on ring 3, 11; 80+ rings</t>
+  </si>
+  <si>
+    <t>check ring 15 (another ring?); 80+ rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> check ring 52 (unsure ring or crack); ring 60 hard to decipher ring boundary; check ring 62 (crack); check crack on ring 65; 80+ rings</t>
+  </si>
+  <si>
+    <t>some parts were quite wavy; 80+ rings</t>
+  </si>
+  <si>
+    <t>Check rings 5-8 (wavy/rotting?); super wavy; crack between rings 39-41; check ring 43; 80+ rings</t>
+  </si>
+  <si>
+    <t>ring 31 was wavy; check ring 52 (some parts looked like 2 rings); 80+ rings</t>
+  </si>
+  <si>
+    <t>check ring 40/41, 48-51, 55, 77-80; I am very confused with the ring boundaries on this one; 80+ rings</t>
+  </si>
+  <si>
+    <t>missing??</t>
+  </si>
+  <si>
+    <t>check ring 18 (dust covering ring boundary); 80+ rings</t>
+  </si>
+  <si>
+    <t>fixed crack on 63; 80+ rings</t>
+  </si>
+  <si>
+    <t>dust covering ring 57/8, fixed crack on 61; check ring 77; 80+ rings</t>
+  </si>
+  <si>
+    <t>light inner bark noted; check ring 49 (lots of dust); check ring 63; 80+ rings</t>
+  </si>
+  <si>
+    <t>ring 19 fixed crack or dust; 80+ rings</t>
+  </si>
+  <si>
+    <t>crack on ring 7 (partially filled?)</t>
+  </si>
+  <si>
+    <t>check ring 69; 80+ rings</t>
+  </si>
+  <si>
+    <t>crack b/w ring 6-8; 80+ rings</t>
+  </si>
+  <si>
+    <t>small crack on ring 8; check ring 69; 80+ rings</t>
+  </si>
+  <si>
+    <t>80+ ring</t>
+  </si>
+  <si>
+    <t>check rings 11-12, fixed crack on ring 17, check ring 45; 80+ rings</t>
+  </si>
+  <si>
+    <t>check ring 17 (large filled crack); check ring 35 (small embedded ring?); check ring 57 (crack split rings); 80+ rings</t>
+  </si>
+  <si>
+    <t>some regions hard to decipher, very blurry</t>
+  </si>
+  <si>
+    <t>check rings 48 &amp; 51 (are ring boundaries correct? Some very small); 80+ rings</t>
+  </si>
+  <si>
+    <t>disjointed at ring 9/10- check; check rings 44-46 (crack across); 80+ rings</t>
+  </si>
+  <si>
+    <t>check ring 16; 80+ rings</t>
+  </si>
+  <si>
+    <t>go over rings 1-6 (blurry and tiny); had to measure from edge of core (super washed out)</t>
+  </si>
+  <si>
+    <t>check rings 1-3 (very blurry); check ring 6&amp;9 - actual rings? (very small); not very confident about this core; check ring 40 (colour division in earlywood); 80+ rings</t>
+  </si>
+  <si>
+    <t>check ring 4; check ring 8 (very small not sure); check ring 38 (same reason); check ring 48 (embedded ring?); crack on ring 73; 80+ rings</t>
+  </si>
+  <si>
+    <t>crack on ring 36 (filled in); crack on 78 (I went around it); 80+ rings</t>
+  </si>
+  <si>
+    <t>tip missing; ring 39 - some parts have defined latewood, others fade into ring 38; 80+ rings</t>
+  </si>
+  <si>
+    <t>don’t know if ring 66 boundary is correct (is it latewoor/smthn else?); 80+ rings</t>
+  </si>
+  <si>
+    <t>ring 69 unclear boundary; 80+ rings</t>
+  </si>
+  <si>
+    <t>filled crack on ring 24; very blurry around ring 68-70; 80+ rings</t>
+  </si>
+  <si>
+    <t>very blurry- did not complete</t>
+  </si>
+  <si>
+    <t>very blurry especially first few rings - review; ring 32 (not a complete ring across?); check ring 46-50 (unsure of ring boundaries); I gave up at ring 64</t>
+  </si>
+  <si>
+    <t>blurry-review rings 1-5, 25; 80+ rings</t>
+  </si>
+  <si>
+    <t>check ring 35 (it is a small ring or part of other ring latewood?); 80+ rings</t>
+  </si>
+  <si>
+    <t>filled crack ring4; check ring 17; 80+ ring</t>
+  </si>
+  <si>
+    <t>check start of core (inner bark?); stopped at 51 - difficult to decipher ring boundaries</t>
   </si>
 </sst>
 </file>
@@ -4134,6 +4313,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6988,7 +7171,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BC15E8E-B068-4223-8546-CDE134FBDB67}">
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="4" max="4" width="11.36328125" customWidth="1"/>
@@ -7028,6 +7211,18 @@
       <c r="C2" t="s">
         <v>115</v>
       </c>
+      <c r="D2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E2" s="5">
+        <v>46203</v>
+      </c>
+      <c r="F2">
+        <v>80</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1258</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -7039,6 +7234,18 @@
       <c r="C3" t="s">
         <v>115</v>
       </c>
+      <c r="D3" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46203</v>
+      </c>
+      <c r="F3">
+        <v>80</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1257</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -7050,6 +7257,18 @@
       <c r="C4" t="s">
         <v>115</v>
       </c>
+      <c r="D4" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E4" s="5">
+        <v>46203</v>
+      </c>
+      <c r="F4">
+        <v>80</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -7061,6 +7280,18 @@
       <c r="C5" t="s">
         <v>115</v>
       </c>
+      <c r="D5" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E5" s="5">
+        <v>46203</v>
+      </c>
+      <c r="F5">
+        <v>80</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1259</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -7072,6 +7303,18 @@
       <c r="C6" t="s">
         <v>115</v>
       </c>
+      <c r="D6" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E6" s="5">
+        <v>46205</v>
+      </c>
+      <c r="F6">
+        <v>80</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1256</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -7083,6 +7326,18 @@
       <c r="C7" t="s">
         <v>115</v>
       </c>
+      <c r="D7" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E7" s="5">
+        <v>46205</v>
+      </c>
+      <c r="F7">
+        <v>80</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1255</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -7094,6 +7349,18 @@
       <c r="C8" t="s">
         <v>115</v>
       </c>
+      <c r="D8" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E8" s="5">
+        <v>46206</v>
+      </c>
+      <c r="F8">
+        <v>80</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -7105,6 +7372,18 @@
       <c r="C9" t="s">
         <v>115</v>
       </c>
+      <c r="D9" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E9" s="5">
+        <v>46206</v>
+      </c>
+      <c r="F9">
+        <v>80</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1261</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -7116,6 +7395,18 @@
       <c r="C10" t="s">
         <v>115</v>
       </c>
+      <c r="D10" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E10" s="5">
+        <v>46206</v>
+      </c>
+      <c r="F10">
+        <v>80</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1260</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -7127,8 +7418,17 @@
       <c r="C11" t="s">
         <v>115</v>
       </c>
+      <c r="D11" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E11" s="5">
+        <v>46210</v>
+      </c>
+      <c r="F11">
+        <v>80</v>
+      </c>
       <c r="G11" t="s">
-        <v>1242</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -7141,6 +7441,18 @@
       <c r="C12" t="s">
         <v>115</v>
       </c>
+      <c r="D12" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E12" s="5">
+        <v>46210</v>
+      </c>
+      <c r="F12">
+        <v>80</v>
+      </c>
+      <c r="G12" t="s">
+        <v>1263</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
@@ -7152,6 +7464,18 @@
       <c r="C13" t="s">
         <v>115</v>
       </c>
+      <c r="D13" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E13" s="5">
+        <v>46211</v>
+      </c>
+      <c r="F13">
+        <v>80</v>
+      </c>
+      <c r="G13" t="s">
+        <v>1264</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
@@ -7163,6 +7487,18 @@
       <c r="C14" t="s">
         <v>115</v>
       </c>
+      <c r="D14" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E14" s="5">
+        <v>46211</v>
+      </c>
+      <c r="F14">
+        <v>80</v>
+      </c>
+      <c r="G14" t="s">
+        <v>1265</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
@@ -7174,6 +7510,18 @@
       <c r="C15" t="s">
         <v>115</v>
       </c>
+      <c r="D15" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E15" s="5">
+        <v>46211</v>
+      </c>
+      <c r="F15">
+        <v>80</v>
+      </c>
+      <c r="G15" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
@@ -7185,8 +7533,20 @@
       <c r="C16" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="D16" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E16" s="5">
+        <v>46211</v>
+      </c>
+      <c r="F16">
+        <v>80</v>
+      </c>
+      <c r="G16" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>218</v>
       </c>
@@ -7196,8 +7556,20 @@
       <c r="C17" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
+      <c r="D17" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E17" s="5">
+        <v>46211</v>
+      </c>
+      <c r="F17">
+        <v>80</v>
+      </c>
+      <c r="G17" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>218</v>
       </c>
@@ -7207,8 +7579,20 @@
       <c r="C18" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="D18" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E18" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F18">
+        <v>80</v>
+      </c>
+      <c r="G18" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>218</v>
       </c>
@@ -7218,8 +7602,20 @@
       <c r="C19" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
+      <c r="D19" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E19" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F19">
+        <v>80</v>
+      </c>
+      <c r="G19" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>218</v>
       </c>
@@ -7229,8 +7625,20 @@
       <c r="C20" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
+      <c r="D20" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E20" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F20">
+        <v>80</v>
+      </c>
+      <c r="G20" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>218</v>
       </c>
@@ -7240,8 +7648,20 @@
       <c r="C21" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="22" spans="1:3">
+      <c r="D21" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E21" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F21">
+        <v>80</v>
+      </c>
+      <c r="G21" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>218</v>
       </c>
@@ -7251,8 +7671,20 @@
       <c r="C22" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="23" spans="1:3">
+      <c r="D22" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E22" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F22">
+        <v>80</v>
+      </c>
+      <c r="G22" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>218</v>
       </c>
@@ -7262,8 +7694,20 @@
       <c r="C23" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="24" spans="1:3">
+      <c r="D23" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E23" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F23">
+        <v>80</v>
+      </c>
+      <c r="G23" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>218</v>
       </c>
@@ -7273,8 +7717,20 @@
       <c r="C24" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="25" spans="1:3">
+      <c r="D24" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E24" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F24">
+        <v>75</v>
+      </c>
+      <c r="G24" t="s">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>218</v>
       </c>
@@ -7284,8 +7740,20 @@
       <c r="C25" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="26" spans="1:3">
+      <c r="D25" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E25" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F25">
+        <v>69</v>
+      </c>
+      <c r="G25" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>218</v>
       </c>
@@ -7295,8 +7763,17 @@
       <c r="C26" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="27" spans="1:3">
+      <c r="D26" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E26" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F26">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>218</v>
       </c>
@@ -7306,8 +7783,17 @@
       <c r="C27" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="28" spans="1:3">
+      <c r="D27" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E27" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F27">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>218</v>
       </c>
@@ -7317,8 +7803,20 @@
       <c r="C28" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="29" spans="1:3">
+      <c r="D28" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E28" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F28">
+        <v>80</v>
+      </c>
+      <c r="G28" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>218</v>
       </c>
@@ -7328,8 +7826,20 @@
       <c r="C29" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="30" spans="1:3">
+      <c r="D29" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E29" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F29">
+        <v>80</v>
+      </c>
+      <c r="G29" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>218</v>
       </c>
@@ -7339,8 +7849,20 @@
       <c r="C30" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="31" spans="1:3">
+      <c r="D30" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E30" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F30">
+        <v>80</v>
+      </c>
+      <c r="G30" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>218</v>
       </c>
@@ -7350,8 +7872,17 @@
       <c r="C31" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="32" spans="1:3">
+      <c r="D31" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E31" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F31">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>218</v>
       </c>
@@ -7361,8 +7892,20 @@
       <c r="C32" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="33" spans="1:3">
+      <c r="D32" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E32" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F32">
+        <v>80</v>
+      </c>
+      <c r="G32" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>218</v>
       </c>
@@ -7372,8 +7915,20 @@
       <c r="C33" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="D33" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E33" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F33">
+        <v>80</v>
+      </c>
+      <c r="G33" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>218</v>
       </c>
@@ -7383,8 +7938,20 @@
       <c r="C34" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="D34" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E34" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F34">
+        <v>80</v>
+      </c>
+      <c r="G34" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>218</v>
       </c>
@@ -7394,8 +7961,20 @@
       <c r="C35" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="36" spans="1:3">
+      <c r="D35" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E35" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F35">
+        <v>80</v>
+      </c>
+      <c r="G35" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>218</v>
       </c>
@@ -7405,8 +7984,20 @@
       <c r="C36" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="37" spans="1:3">
+      <c r="D36" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E36" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F36">
+        <v>80</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>218</v>
       </c>
@@ -7416,8 +8007,20 @@
       <c r="C37" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="38" spans="1:3">
+      <c r="D37" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E37" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F37">
+        <v>80</v>
+      </c>
+      <c r="G37" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>218</v>
       </c>
@@ -7427,8 +8030,20 @@
       <c r="C38" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="39" spans="1:3">
+      <c r="D38" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E38" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F38">
+        <v>80</v>
+      </c>
+      <c r="G38" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>218</v>
       </c>
@@ -7438,8 +8053,20 @@
       <c r="C39" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="40" spans="1:3">
+      <c r="D39" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E39" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F39">
+        <v>80</v>
+      </c>
+      <c r="G39" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>218</v>
       </c>
@@ -7449,8 +8076,20 @@
       <c r="C40" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="41" spans="1:3">
+      <c r="D40" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E40" s="5">
+        <v>46212</v>
+      </c>
+      <c r="F40">
+        <v>80</v>
+      </c>
+      <c r="G40" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>218</v>
       </c>
@@ -7460,8 +8099,20 @@
       <c r="C41" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="42" spans="1:3">
+      <c r="D41" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E41" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F41">
+        <v>80</v>
+      </c>
+      <c r="G41" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>218</v>
       </c>
@@ -7471,8 +8122,20 @@
       <c r="C42" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="43" spans="1:3">
+      <c r="D42" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E42" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F42">
+        <v>80</v>
+      </c>
+      <c r="G42" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>218</v>
       </c>
@@ -7482,8 +8145,20 @@
       <c r="C43" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="44" spans="1:3">
+      <c r="D43" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E43" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F43">
+        <v>80</v>
+      </c>
+      <c r="G43" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>218</v>
       </c>
@@ -7493,8 +8168,20 @@
       <c r="C44" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="45" spans="1:3">
+      <c r="D44" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E44" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F44">
+        <v>80</v>
+      </c>
+      <c r="G44" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>218</v>
       </c>
@@ -7504,8 +8191,20 @@
       <c r="C45" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="46" spans="1:3">
+      <c r="D45" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E45" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F45">
+        <v>80</v>
+      </c>
+      <c r="G45" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>218</v>
       </c>
@@ -7515,8 +8214,20 @@
       <c r="C46" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="47" spans="1:3">
+      <c r="D46" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E46" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F46">
+        <v>80</v>
+      </c>
+      <c r="G46" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>218</v>
       </c>
@@ -7526,8 +8237,20 @@
       <c r="C47" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="48" spans="1:3">
+      <c r="D47" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E47" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F47">
+        <v>80</v>
+      </c>
+      <c r="G47" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>218</v>
       </c>
@@ -7537,8 +8260,20 @@
       <c r="C48" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="49" spans="1:3">
+      <c r="D48" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E48" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F48">
+        <v>80</v>
+      </c>
+      <c r="G48" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
         <v>218</v>
       </c>
@@ -7548,8 +8283,20 @@
       <c r="C49" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
+      <c r="D49" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E49" s="5">
+        <v>46213</v>
+      </c>
+      <c r="F49">
+        <v>80</v>
+      </c>
+      <c r="G49" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>218</v>
       </c>
@@ -7559,8 +8306,20 @@
       <c r="C50" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="51" spans="1:3">
+      <c r="D50" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E50" s="5">
+        <v>46214</v>
+      </c>
+      <c r="F50">
+        <v>80</v>
+      </c>
+      <c r="G50" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>218</v>
       </c>
@@ -7570,8 +8329,20 @@
       <c r="C51" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="52" spans="1:3">
+      <c r="D51" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E51" s="5">
+        <v>46214</v>
+      </c>
+      <c r="F51">
+        <v>80</v>
+      </c>
+      <c r="G51" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>219</v>
       </c>
@@ -7581,8 +8352,11 @@
       <c r="C52" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
+      <c r="D52" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
         <v>218</v>
       </c>
@@ -7592,8 +8366,20 @@
       <c r="C53" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="54" spans="1:3">
+      <c r="D53" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E53" s="5">
+        <v>46214</v>
+      </c>
+      <c r="F53">
+        <v>80</v>
+      </c>
+      <c r="G53" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>218</v>
       </c>
@@ -7603,8 +8389,20 @@
       <c r="C54" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="55" spans="1:3">
+      <c r="D54" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E54" s="5">
+        <v>46214</v>
+      </c>
+      <c r="F54">
+        <v>80</v>
+      </c>
+      <c r="G54" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
         <v>218</v>
       </c>
@@ -7614,8 +8412,20 @@
       <c r="C55" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="56" spans="1:3">
+      <c r="D55" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E55" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F55">
+        <v>80</v>
+      </c>
+      <c r="G55" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>218</v>
       </c>
@@ -7625,8 +8435,20 @@
       <c r="C56" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
+      <c r="D56" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E56" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F56">
+        <v>80</v>
+      </c>
+      <c r="G56" t="s">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>218</v>
       </c>
@@ -7636,8 +8458,20 @@
       <c r="C57" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="58" spans="1:3">
+      <c r="D57" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E57" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F57">
+        <v>80</v>
+      </c>
+      <c r="G57" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>218</v>
       </c>
@@ -7647,8 +8481,20 @@
       <c r="C58" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="59" spans="1:3">
+      <c r="D58" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E58" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F58">
+        <v>80</v>
+      </c>
+      <c r="G58" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>218</v>
       </c>
@@ -7658,8 +8504,20 @@
       <c r="C59" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="60" spans="1:3">
+      <c r="D59" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E59" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F59">
+        <v>80</v>
+      </c>
+      <c r="G59" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>218</v>
       </c>
@@ -7669,8 +8527,20 @@
       <c r="C60" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="61" spans="1:3">
+      <c r="D60" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E60" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F60">
+        <v>80</v>
+      </c>
+      <c r="G60" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
         <v>218</v>
       </c>
@@ -7680,8 +8550,20 @@
       <c r="C61" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
+      <c r="D61" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E61" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F61">
+        <v>51</v>
+      </c>
+      <c r="G61" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
         <v>218</v>
       </c>
@@ -7691,8 +8573,20 @@
       <c r="C62" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="63" spans="1:3">
+      <c r="D62" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E62" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F62">
+        <v>80</v>
+      </c>
+      <c r="G62" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
         <v>218</v>
       </c>
@@ -7702,8 +8596,20 @@
       <c r="C63" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="64" spans="1:3">
+      <c r="D63" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E63" s="5">
+        <v>46215</v>
+      </c>
+      <c r="F63">
+        <v>80</v>
+      </c>
+      <c r="G63" t="s">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
         <v>218</v>
       </c>
@@ -7713,8 +8619,20 @@
       <c r="C64" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="65" spans="1:7">
+      <c r="D64" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E64" s="5">
+        <v>46239</v>
+      </c>
+      <c r="F64">
+        <v>80</v>
+      </c>
+      <c r="G64" t="s">
+        <v>1283</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
       <c r="A65" t="s">
         <v>218</v>
       </c>
@@ -7724,8 +8642,20 @@
       <c r="C65" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="66" spans="1:7">
+      <c r="D65" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E65" s="5">
+        <v>46239</v>
+      </c>
+      <c r="F65">
+        <v>67</v>
+      </c>
+      <c r="G65" t="s">
+        <v>1284</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
       <c r="A66" t="s">
         <v>218</v>
       </c>
@@ -7735,8 +8665,20 @@
       <c r="C66" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="67" spans="1:7">
+      <c r="D66" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E66" s="5">
+        <v>46239</v>
+      </c>
+      <c r="F66">
+        <v>80</v>
+      </c>
+      <c r="G66" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
       <c r="A67" t="s">
         <v>218</v>
       </c>
@@ -7746,8 +8688,20 @@
       <c r="C67" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="68" spans="1:7">
+      <c r="D67" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E67" s="5">
+        <v>46239</v>
+      </c>
+      <c r="F67">
+        <v>80</v>
+      </c>
+      <c r="G67" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
       <c r="A68" t="s">
         <v>218</v>
       </c>
@@ -7757,8 +8711,20 @@
       <c r="C68" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="69" spans="1:7">
+      <c r="D68" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E68" s="5">
+        <v>46239</v>
+      </c>
+      <c r="F68">
+        <v>80</v>
+      </c>
+      <c r="G68" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
       <c r="A69" t="s">
         <v>218</v>
       </c>
@@ -7768,8 +8734,20 @@
       <c r="C69" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="70" spans="1:7">
+      <c r="D69" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E69" s="5">
+        <v>46244</v>
+      </c>
+      <c r="F69">
+        <v>80</v>
+      </c>
+      <c r="G69" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
       <c r="A70" t="s">
         <v>218</v>
       </c>
@@ -7779,30 +8757,48 @@
       <c r="C70" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="71" spans="1:7">
+      <c r="D70" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E70" s="5">
+        <v>46244</v>
+      </c>
+      <c r="F70">
+        <v>80</v>
+      </c>
+      <c r="G70" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
       <c r="A71" t="s">
         <v>218</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="1" t="s">
         <v>222</v>
       </c>
       <c r="C71" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="72" spans="1:7">
+      <c r="D71" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
       <c r="A72" t="s">
         <v>218</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="1" t="s">
         <v>223</v>
       </c>
       <c r="C72" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="73" spans="1:7">
+      <c r="D72" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
       <c r="A73" t="s">
         <v>218</v>
       </c>
@@ -7812,8 +8808,20 @@
       <c r="C73" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="74" spans="1:7">
+      <c r="D73" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E73" s="5">
+        <v>46244</v>
+      </c>
+      <c r="F73">
+        <v>80</v>
+      </c>
+      <c r="G73" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
       <c r="A74" t="s">
         <v>218</v>
       </c>
@@ -7823,8 +8831,20 @@
       <c r="C74" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="75" spans="1:7">
+      <c r="D74" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E74" s="5">
+        <v>46244</v>
+      </c>
+      <c r="F74">
+        <v>80</v>
+      </c>
+      <c r="G74" t="s">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
       <c r="A75" t="s">
         <v>218</v>
       </c>
@@ -7834,8 +8854,20 @@
       <c r="C75" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="76" spans="1:7">
+      <c r="D75" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E75" s="5">
+        <v>46244</v>
+      </c>
+      <c r="F75">
+        <v>80</v>
+      </c>
+      <c r="G75" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
       <c r="A76" t="s">
         <v>218</v>
       </c>
@@ -7845,33 +8877,51 @@
       <c r="C76" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="77" spans="1:7">
+      <c r="D76" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E76" s="5">
+        <v>46244</v>
+      </c>
+      <c r="F76">
+        <v>80</v>
+      </c>
+      <c r="G76" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
       <c r="A77" t="s">
         <v>219</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="1" t="s">
         <v>224</v>
       </c>
       <c r="C77" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="78" spans="1:7">
+      <c r="D77" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
       <c r="A78" t="s">
         <v>219</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="1" t="s">
         <v>225</v>
       </c>
       <c r="C78" t="s">
         <v>116</v>
       </c>
+      <c r="D78" t="s">
+        <v>1278</v>
+      </c>
       <c r="G78" t="s">
         <v>1242</v>
       </c>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:8">
       <c r="A79" t="s">
         <v>218</v>
       </c>
@@ -7881,16 +8931,34 @@
       <c r="C79" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="80" spans="1:7">
+      <c r="D79" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E79" s="5">
+        <v>46245</v>
+      </c>
+      <c r="F79">
+        <v>80</v>
+      </c>
+      <c r="G79" t="s">
+        <v>1253</v>
+      </c>
+      <c r="H79" t="s">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
       <c r="A80" t="s">
         <v>218</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="1" t="s">
         <v>214</v>
       </c>
       <c r="C80" t="s">
         <v>116</v>
+      </c>
+      <c r="G80" t="s">
+        <v>1303</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -7903,6 +8971,18 @@
       <c r="C81" t="s">
         <v>116</v>
       </c>
+      <c r="D81" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E81" s="5">
+        <v>46245</v>
+      </c>
+      <c r="F81">
+        <v>80</v>
+      </c>
+      <c r="G81" t="s">
+        <v>1292</v>
+      </c>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" t="s">
@@ -7914,6 +8994,18 @@
       <c r="C82" t="s">
         <v>116</v>
       </c>
+      <c r="D82" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E82" s="5">
+        <v>46245</v>
+      </c>
+      <c r="F82">
+        <v>80</v>
+      </c>
+      <c r="G82" t="s">
+        <v>1293</v>
+      </c>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" t="s">
@@ -7925,6 +9017,18 @@
       <c r="C83" t="s">
         <v>116</v>
       </c>
+      <c r="D83" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E83" s="5">
+        <v>46245</v>
+      </c>
+      <c r="F83">
+        <v>80</v>
+      </c>
+      <c r="G83" t="s">
+        <v>1294</v>
+      </c>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" t="s">
@@ -7936,6 +9040,18 @@
       <c r="C84" t="s">
         <v>116</v>
       </c>
+      <c r="D84" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E84" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F84">
+        <v>80</v>
+      </c>
+      <c r="G84" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="85" spans="1:7">
       <c r="A85" t="s">
@@ -7947,6 +9063,18 @@
       <c r="C85" t="s">
         <v>116</v>
       </c>
+      <c r="D85" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E85" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F85">
+        <v>80</v>
+      </c>
+      <c r="G85" t="s">
+        <v>1295</v>
+      </c>
     </row>
     <row r="86" spans="1:7">
       <c r="A86" t="s">
@@ -7958,6 +9086,18 @@
       <c r="C86" t="s">
         <v>116</v>
       </c>
+      <c r="D86" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E86" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F86">
+        <v>80</v>
+      </c>
+      <c r="G86" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="87" spans="1:7">
       <c r="A87" t="s">
@@ -7969,6 +9109,18 @@
       <c r="C87" t="s">
         <v>116</v>
       </c>
+      <c r="D87" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E87" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F87">
+        <v>80</v>
+      </c>
+      <c r="G87" t="s">
+        <v>1296</v>
+      </c>
     </row>
     <row r="88" spans="1:7">
       <c r="A88" t="s">
@@ -7980,6 +9132,18 @@
       <c r="C88" t="s">
         <v>116</v>
       </c>
+      <c r="D88" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E88" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F88">
+        <v>80</v>
+      </c>
+      <c r="G88" t="s">
+        <v>1297</v>
+      </c>
     </row>
     <row r="89" spans="1:7">
       <c r="A89" t="s">
@@ -7991,6 +9155,18 @@
       <c r="C89" t="s">
         <v>116</v>
       </c>
+      <c r="D89" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E89" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F89">
+        <v>80</v>
+      </c>
+      <c r="G89" t="s">
+        <v>1298</v>
+      </c>
     </row>
     <row r="90" spans="1:7">
       <c r="A90" t="s">
@@ -8002,8 +9178,17 @@
       <c r="C90" t="s">
         <v>116</v>
       </c>
+      <c r="D90" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E90" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F90">
+        <v>80</v>
+      </c>
       <c r="G90" t="s">
-        <v>1242</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -8016,6 +9201,18 @@
       <c r="C91" t="s">
         <v>116</v>
       </c>
+      <c r="D91" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E91" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F91">
+        <v>80</v>
+      </c>
+      <c r="G91" t="s">
+        <v>1300</v>
+      </c>
     </row>
     <row r="92" spans="1:7">
       <c r="A92" t="s">
@@ -8027,6 +9224,18 @@
       <c r="C92" t="s">
         <v>116</v>
       </c>
+      <c r="D92" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E92" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F92">
+        <v>80</v>
+      </c>
+      <c r="G92" t="s">
+        <v>1301</v>
+      </c>
     </row>
     <row r="93" spans="1:7">
       <c r="A93" t="s">
@@ -8038,6 +9247,18 @@
       <c r="C93" t="s">
         <v>116</v>
       </c>
+      <c r="D93" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E93" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F93">
+        <v>80</v>
+      </c>
+      <c r="G93" t="s">
+        <v>1302</v>
+      </c>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" t="s">
@@ -8049,6 +9270,18 @@
       <c r="C94" t="s">
         <v>116</v>
       </c>
+      <c r="D94" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E94" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F94">
+        <v>64</v>
+      </c>
+      <c r="G94" t="s">
+        <v>1304</v>
+      </c>
     </row>
     <row r="95" spans="1:7">
       <c r="A95" t="s">
@@ -8060,16 +9293,31 @@
       <c r="C95" t="s">
         <v>116</v>
       </c>
+      <c r="D95" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E95" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F95">
+        <v>80</v>
+      </c>
+      <c r="G95" t="s">
+        <v>1305</v>
+      </c>
     </row>
     <row r="96" spans="1:7">
       <c r="A96" t="s">
         <v>219</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="1" t="s">
         <v>226</v>
       </c>
       <c r="C96" t="s">
         <v>116</v>
+      </c>
+      <c r="D96" t="s">
+        <v>1278</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -8082,6 +9330,18 @@
       <c r="C97" t="s">
         <v>116</v>
       </c>
+      <c r="D97" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E97" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F97">
+        <v>80</v>
+      </c>
+      <c r="G97" t="s">
+        <v>1306</v>
+      </c>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" t="s">
@@ -8093,27 +9353,45 @@
       <c r="C98" t="s">
         <v>116</v>
       </c>
+      <c r="D98" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E98" s="5">
+        <v>46246</v>
+      </c>
+      <c r="F98">
+        <v>80</v>
+      </c>
+      <c r="G98" t="s">
+        <v>1307</v>
+      </c>
     </row>
     <row r="99" spans="1:7">
       <c r="A99" t="s">
         <v>219</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="1" t="s">
         <v>227</v>
       </c>
       <c r="C99" t="s">
         <v>116</v>
+      </c>
+      <c r="D99" t="s">
+        <v>1278</v>
       </c>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" t="s">
         <v>219</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="1" t="s">
         <v>228</v>
       </c>
       <c r="C100" t="s">
         <v>116</v>
+      </c>
+      <c r="D100" t="s">
+        <v>1278</v>
       </c>
     </row>
     <row r="101" spans="1:7">
@@ -8126,6 +9404,18 @@
       <c r="C101" t="s">
         <v>217</v>
       </c>
+      <c r="D101" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E101" s="5">
+        <v>46182</v>
+      </c>
+      <c r="F101">
+        <v>80</v>
+      </c>
+      <c r="G101" t="s">
+        <v>1252</v>
+      </c>
     </row>
     <row r="102" spans="1:7">
       <c r="A102" t="s">
@@ -8141,13 +9431,13 @@
         <v>1251</v>
       </c>
       <c r="E102" s="5">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="F102">
-        <v>153</v>
+        <v>80</v>
       </c>
       <c r="G102" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="103" spans="1:7">
@@ -8160,6 +9450,18 @@
       <c r="C103" t="s">
         <v>217</v>
       </c>
+      <c r="D103" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E103" s="5">
+        <v>46184</v>
+      </c>
+      <c r="F103">
+        <v>80</v>
+      </c>
+      <c r="G103" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" t="s">
@@ -8171,6 +9473,18 @@
       <c r="C104" t="s">
         <v>217</v>
       </c>
+      <c r="D104" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E104" s="5">
+        <v>46185</v>
+      </c>
+      <c r="F104">
+        <v>80</v>
+      </c>
+      <c r="G104" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="105" spans="1:7">
       <c r="A105" t="s">
@@ -8182,6 +9496,18 @@
       <c r="C105" t="s">
         <v>217</v>
       </c>
+      <c r="D105" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E105" s="5">
+        <v>46185</v>
+      </c>
+      <c r="F105">
+        <v>80</v>
+      </c>
+      <c r="G105" t="s">
+        <v>1253</v>
+      </c>
     </row>
     <row r="106" spans="1:7">
       <c r="A106" t="s">
@@ -8192,6 +9518,18 @@
       </c>
       <c r="C106" t="s">
         <v>217</v>
+      </c>
+      <c r="D106" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E106" s="5">
+        <v>46203</v>
+      </c>
+      <c r="F106">
+        <v>80</v>
+      </c>
+      <c r="G106" t="s">
+        <v>1253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
completed TSHE rings from SUNR
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned_Brahmleen.xlsx
+++ b/notes/coreMeasurement/coresScanned_Brahmleen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangxm29.stu\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77DDC8A-3FA6-4D13-B206-1AC91D707A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6AB003-01EC-4A1D-9273-F1FC2EB774F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4051" uniqueCount="1328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4070" uniqueCount="1335">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4295,6 +4295,27 @@
   </si>
   <si>
     <t>start point unclear; dusty- ring boundaries bit fuzzy</t>
+  </si>
+  <si>
+    <t>frost marks on ring 11, 115-119; 130+</t>
+  </si>
+  <si>
+    <t>frost marks on ring 23, 28; 130+</t>
+  </si>
+  <si>
+    <t>very dusty all over; crack on ring 87, 97, 113, 114 &amp; 119; frost marks on ring 94; 130+</t>
+  </si>
+  <si>
+    <t>130+; blurry</t>
+  </si>
+  <si>
+    <t>130+; blurry; frost marks on ring 19; blurry and dusty check if ring 60 is an actual ring</t>
+  </si>
+  <si>
+    <t>crack on ring 8</t>
+  </si>
+  <si>
+    <t>frost  marks on ring 26</t>
   </si>
 </sst>
 </file>
@@ -17558,7 +17579,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C353DFE2-926D-4FA7-B43B-F35C7CA7AB01}">
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="3" width="8.6328125" style="2"/>
@@ -18283,7 +18304,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:8">
       <c r="A65" s="2" t="s">
         <v>933</v>
       </c>
@@ -18294,7 +18315,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:8">
       <c r="A66" s="2" t="s">
         <v>933</v>
       </c>
@@ -18305,7 +18326,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:8">
       <c r="A67" s="2" t="s">
         <v>933</v>
       </c>
@@ -18316,7 +18337,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:8">
       <c r="A68" s="2" t="s">
         <v>933</v>
       </c>
@@ -18327,7 +18348,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:8">
       <c r="A69" s="2" t="s">
         <v>933</v>
       </c>
@@ -18338,7 +18359,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:8">
       <c r="A70" s="2" t="s">
         <v>933</v>
       </c>
@@ -18349,7 +18370,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:8">
       <c r="A71" s="2" t="s">
         <v>933</v>
       </c>
@@ -18360,7 +18381,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:8">
       <c r="A72" s="2" t="s">
         <v>933</v>
       </c>
@@ -18371,7 +18392,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:8">
       <c r="A73" s="2" t="s">
         <v>933</v>
       </c>
@@ -18382,7 +18403,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:8">
       <c r="A74" s="2" t="s">
         <v>933</v>
       </c>
@@ -18393,7 +18414,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:8">
       <c r="A75" s="2" t="s">
         <v>933</v>
       </c>
@@ -18403,8 +18424,20 @@
       <c r="C75" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="76" spans="1:3">
+      <c r="D75" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E75" s="5">
+        <v>46260</v>
+      </c>
+      <c r="F75" s="2">
+        <v>130</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
       <c r="A76" s="2" t="s">
         <v>933</v>
       </c>
@@ -18414,8 +18447,20 @@
       <c r="C76" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="77" spans="1:3">
+      <c r="D76" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E76" s="5">
+        <v>46260</v>
+      </c>
+      <c r="F76">
+        <v>130</v>
+      </c>
+      <c r="G76" t="s">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
       <c r="A77" s="2" t="s">
         <v>933</v>
       </c>
@@ -18425,8 +18470,20 @@
       <c r="C77" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="78" spans="1:3">
+      <c r="D77" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E77" s="5">
+        <v>46260</v>
+      </c>
+      <c r="F77">
+        <v>130</v>
+      </c>
+      <c r="G77" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
       <c r="A78" s="2" t="s">
         <v>933</v>
       </c>
@@ -18436,8 +18493,20 @@
       <c r="C78" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="79" spans="1:3">
+      <c r="D78" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E78" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F78">
+        <v>130</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
       <c r="A79" s="2" t="s">
         <v>933</v>
       </c>
@@ -18447,8 +18516,21 @@
       <c r="C79" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="80" spans="1:3">
+      <c r="D79" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E79" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F79">
+        <v>130</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>1331</v>
+      </c>
+      <c r="H79" s="2"/>
+    </row>
+    <row r="80" spans="1:8">
       <c r="A80" s="2" t="s">
         <v>933</v>
       </c>
@@ -18457,6 +18539,18 @@
       </c>
       <c r="C80" s="2" t="s">
         <v>361</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E80" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F80">
+        <v>130</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>1332</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -18469,6 +18563,18 @@
       <c r="C81" s="2" t="s">
         <v>361</v>
       </c>
+      <c r="D81" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E81" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F81">
+        <v>80</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>1309</v>
+      </c>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" s="2" t="s">
@@ -18480,6 +18586,15 @@
       <c r="C82" s="2" t="s">
         <v>361</v>
       </c>
+      <c r="D82" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E82" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F82">
+        <v>81</v>
+      </c>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="2" t="s">
@@ -18491,6 +18606,18 @@
       <c r="C83" s="2" t="s">
         <v>361</v>
       </c>
+      <c r="D83" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E83" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F83">
+        <v>99</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>1333</v>
+      </c>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" s="2" t="s">
@@ -18501,6 +18628,18 @@
       </c>
       <c r="C84" s="2" t="s">
         <v>361</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E84" s="5">
+        <v>46261</v>
+      </c>
+      <c r="F84">
+        <v>97</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>1334</v>
       </c>
     </row>
     <row r="85" spans="1:7">

</xml_diff>

<commit_message>
CANO measurements for SUNR
</commit_message>
<xml_diff>
--- a/notes/coreMeasurement/coresScanned_Brahmleen.xlsx
+++ b/notes/coreMeasurement/coresScanned_Brahmleen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wangxm29.stu\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6AB003-01EC-4A1D-9273-F1FC2EB774F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CE44A1-621A-4994-B3EB-BB267D35864F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4070" uniqueCount="1335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4124" uniqueCount="1350">
   <si>
     <t>Stand</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -4316,13 +4316,58 @@
   </si>
   <si>
     <t>frost  marks on ring 26</t>
+  </si>
+  <si>
+    <t>rings 75-80 &amp; 120-130 are quite blurry/dusty; 130+</t>
+  </si>
+  <si>
+    <t>check ring 75 (blurry/unsure of boundary); check ring 116 (early wood covered with dust); 130+</t>
+  </si>
+  <si>
+    <t>first few rings are hard to decipher; skipped</t>
+  </si>
+  <si>
+    <t>super faint; skipped</t>
+  </si>
+  <si>
+    <t>faint rings around 59/60; 130+</t>
+  </si>
+  <si>
+    <t>130+; not sure why its highlighted (no cracks)</t>
+  </si>
+  <si>
+    <t>130+; some regions were blurry</t>
+  </si>
+  <si>
+    <t>crack on ring 6; 130+</t>
+  </si>
+  <si>
+    <t>last few rings are a bit blurry; 130+</t>
+  </si>
+  <si>
+    <t>rings undecipherable after 43</t>
+  </si>
+  <si>
+    <t>rings undecipherable after 27</t>
+  </si>
+  <si>
+    <t>hard to decipher rings</t>
+  </si>
+  <si>
+    <t>hard to decipher rings; couldn’t see much after ring 127</t>
+  </si>
+  <si>
+    <t>check ring 26, 101, 105 (another ring?)- super blurry and dusty just review it all</t>
+  </si>
+  <si>
+    <t>frost marks on ring 68; 130+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4335,6 +4380,12 @@
       <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -4364,7 +4415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4377,6 +4428,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17952,7 +18012,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:7">
       <c r="A33" s="2" t="s">
         <v>933</v>
       </c>
@@ -17963,7 +18023,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:7">
       <c r="A34" s="2" t="s">
         <v>933</v>
       </c>
@@ -17974,7 +18034,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:7">
       <c r="A35" s="2" t="s">
         <v>933</v>
       </c>
@@ -17985,7 +18045,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:7">
       <c r="A36" s="2" t="s">
         <v>933</v>
       </c>
@@ -17996,7 +18056,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:7">
       <c r="A37" s="2" t="s">
         <v>933</v>
       </c>
@@ -18007,7 +18067,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:7">
       <c r="A38" s="2" t="s">
         <v>933</v>
       </c>
@@ -18018,7 +18078,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:7">
       <c r="A39" s="2" t="s">
         <v>933</v>
       </c>
@@ -18029,7 +18089,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:7">
       <c r="A40" s="2" t="s">
         <v>933</v>
       </c>
@@ -18040,7 +18100,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:7">
       <c r="A41" s="2" t="s">
         <v>933</v>
       </c>
@@ -18051,7 +18111,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:7">
       <c r="A42" s="2" t="s">
         <v>933</v>
       </c>
@@ -18062,7 +18122,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:7">
       <c r="A43" s="2" t="s">
         <v>933</v>
       </c>
@@ -18073,7 +18133,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:7">
       <c r="A44" s="2" t="s">
         <v>933</v>
       </c>
@@ -18084,7 +18144,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:7">
       <c r="A45" s="2" t="s">
         <v>933</v>
       </c>
@@ -18095,7 +18155,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:7">
       <c r="A46" s="2" t="s">
         <v>933</v>
       </c>
@@ -18105,8 +18165,20 @@
       <c r="C46" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="47" spans="1:3">
+      <c r="D46" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E46" s="5">
+        <v>46262</v>
+      </c>
+      <c r="F46">
+        <v>130</v>
+      </c>
+      <c r="G46" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" s="2" t="s">
         <v>933</v>
       </c>
@@ -18116,8 +18188,20 @@
       <c r="C47" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="48" spans="1:3">
+      <c r="D47" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E47" s="5">
+        <v>46262</v>
+      </c>
+      <c r="F47">
+        <v>130</v>
+      </c>
+      <c r="G47" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" s="2" t="s">
         <v>933</v>
       </c>
@@ -18127,8 +18211,20 @@
       <c r="C48" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="49" spans="1:3">
+      <c r="D48" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E48" s="5">
+        <v>46262</v>
+      </c>
+      <c r="F48">
+        <v>130</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" s="2" t="s">
         <v>933</v>
       </c>
@@ -18138,8 +18234,20 @@
       <c r="C49" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="50" spans="1:3">
+      <c r="D49" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E49" s="5">
+        <v>46262</v>
+      </c>
+      <c r="F49">
+        <v>130</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" s="2" t="s">
         <v>933</v>
       </c>
@@ -18149,8 +18257,20 @@
       <c r="C50" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="51" spans="1:3">
+      <c r="D50" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E50" s="5">
+        <v>46262</v>
+      </c>
+      <c r="F50">
+        <v>130</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" s="2" t="s">
         <v>933</v>
       </c>
@@ -18160,8 +18280,20 @@
       <c r="C51" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="52" spans="1:3">
+      <c r="D51" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E51" s="5">
+        <v>46262</v>
+      </c>
+      <c r="F51">
+        <v>130</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" s="2" t="s">
         <v>933</v>
       </c>
@@ -18171,8 +18303,17 @@
       <c r="C52" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
+      <c r="D52" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E52" s="5">
+        <v>46263</v>
+      </c>
+      <c r="F52">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" s="2" t="s">
         <v>933</v>
       </c>
@@ -18182,9 +18323,18 @@
       <c r="C53" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="54" spans="1:3">
-      <c r="A54" s="2" t="s">
+      <c r="D53" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E53" s="5">
+        <v>46263</v>
+      </c>
+      <c r="F53">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" s="7" t="s">
         <v>933</v>
       </c>
       <c r="B54" s="2" t="s">
@@ -18193,9 +18343,12 @@
       <c r="C54" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" s="2" t="s">
+      <c r="G54" s="2" t="s">
+        <v>1338</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" s="7" t="s">
         <v>933</v>
       </c>
       <c r="B55" s="2" t="s">
@@ -18204,8 +18357,20 @@
       <c r="C55" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="56" spans="1:3">
+      <c r="D55" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E55" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F55">
+        <v>130</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" s="2" t="s">
         <v>933</v>
       </c>
@@ -18215,8 +18380,20 @@
       <c r="C56" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="57" spans="1:3">
+      <c r="D56" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E56" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F56">
+        <v>130</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" s="2" t="s">
         <v>933</v>
       </c>
@@ -18226,8 +18403,11 @@
       <c r="C57" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="58" spans="1:3">
+      <c r="G57" s="2" t="s">
+        <v>1337</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" s="2" t="s">
         <v>933</v>
       </c>
@@ -18237,8 +18417,20 @@
       <c r="C58" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="59" spans="1:3">
+      <c r="D58" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E58" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F58">
+        <v>130</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>1339</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" s="2" t="s">
         <v>933</v>
       </c>
@@ -18248,8 +18440,20 @@
       <c r="C59" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="60" spans="1:3">
+      <c r="D59" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E59" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F59">
+        <v>130</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" s="2" t="s">
         <v>933</v>
       </c>
@@ -18259,8 +18463,20 @@
       <c r="C60" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="61" spans="1:3">
+      <c r="D60" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E60" s="8">
+        <v>46264</v>
+      </c>
+      <c r="F60">
+        <v>130</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>1340</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" s="2" t="s">
         <v>933</v>
       </c>
@@ -18270,8 +18486,20 @@
       <c r="C61" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="62" spans="1:3">
+      <c r="D61" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E61" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F61">
+        <v>130</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" s="2" t="s">
         <v>933</v>
       </c>
@@ -18281,9 +18509,21 @@
       <c r="C62" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" s="2" t="s">
+      <c r="D62" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E62" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F62">
+        <v>130</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>1309</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63" s="6" t="s">
         <v>933</v>
       </c>
       <c r="B63" s="2" t="s">
@@ -18292,8 +18532,20 @@
       <c r="C63" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="64" spans="1:3">
+      <c r="D63" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E63" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F63">
+        <v>130</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" s="2" t="s">
         <v>933</v>
       </c>
@@ -18303,9 +18555,21 @@
       <c r="C64" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D64" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E64" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F64">
+        <v>130</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>1309</v>
+      </c>
     </row>
     <row r="65" spans="1:8">
-      <c r="A65" s="2" t="s">
+      <c r="A65" s="7" t="s">
         <v>933</v>
       </c>
       <c r="B65" s="2" t="s">
@@ -18313,6 +18577,18 @@
       </c>
       <c r="C65" s="2" t="s">
         <v>413</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E65" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F65">
+        <v>130</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>1343</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -18325,6 +18601,18 @@
       <c r="C66" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D66" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E66" s="5">
+        <v>46264</v>
+      </c>
+      <c r="F66">
+        <v>130</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>1309</v>
+      </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" s="2" t="s">
@@ -18336,6 +18624,18 @@
       <c r="C67" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D67" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E67" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F67">
+        <v>43</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>1344</v>
+      </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" s="2" t="s">
@@ -18347,6 +18647,18 @@
       <c r="C68" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D68" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E68" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F68">
+        <v>27</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>1345</v>
+      </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" s="2" t="s">
@@ -18358,6 +18670,18 @@
       <c r="C69" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D69" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E69" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F69">
+        <v>130</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>1346</v>
+      </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" s="2" t="s">
@@ -18369,6 +18693,18 @@
       <c r="C70" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D70" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E70" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F70">
+        <v>127</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>1347</v>
+      </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" s="2" t="s">
@@ -18380,6 +18716,18 @@
       <c r="C71" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D71" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E71" s="8">
+        <v>46265</v>
+      </c>
+      <c r="F71">
+        <v>130</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>1309</v>
+      </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" s="2" t="s">
@@ -18391,6 +18739,18 @@
       <c r="C72" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D72" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E72" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F72">
+        <v>130</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>1348</v>
+      </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" s="2" t="s">
@@ -18402,6 +18762,18 @@
       <c r="C73" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D73" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E73" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F73">
+        <v>130</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>1349</v>
+      </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" s="2" t="s">
@@ -18413,6 +18785,18 @@
       <c r="C74" s="2" t="s">
         <v>413</v>
       </c>
+      <c r="D74" s="2" t="s">
+        <v>1251</v>
+      </c>
+      <c r="E74" s="5">
+        <v>46265</v>
+      </c>
+      <c r="F74">
+        <v>130</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>1309</v>
+      </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" s="2" t="s">
@@ -19314,6 +19698,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>